<commit_message>
SID STAR regression fixed
</commit_message>
<xml_diff>
--- a/Airlines-Services/trajectory/management/commands/SidStar/SID-LIBD-07-PISIP.xlsx
+++ b/Airlines-Services/trajectory/management/commands/SidStar/SID-LIBD-07-PISIP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\Airlines-Services\Airlines-Services\trajectory\management\commands\SidStar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF762FB-4A60-4A3A-B9EB-5FBCD7EB98E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0BA08B-4C54-48A3-911A-FC12998EED0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1280" yWindow="5690" windowWidth="19200" windowHeight="11170" xr2:uid="{5B8640E8-34B0-4460-913B-4CC43B5210E1}"/>
+    <workbookView xWindow="5900" yWindow="3360" windowWidth="15510" windowHeight="11170" xr2:uid="{5B8640E8-34B0-4460-913B-4CC43B5210E1}"/>
   </bookViews>
   <sheets>
     <sheet name="WayPoints" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>order</t>
   </si>
@@ -65,18 +65,12 @@
     <t>LIBD/07</t>
   </si>
   <si>
-    <t>LIBD-07-001</t>
-  </si>
-  <si>
     <t>runway</t>
   </si>
   <si>
     <t>Italy</t>
   </si>
   <si>
-    <t>E16°51'11.30''</t>
-  </si>
-  <si>
     <t>Bari-Rwy-07</t>
   </si>
   <si>
@@ -89,15 +83,6 @@
     <t>Rwy 07</t>
   </si>
   <si>
-    <t>LIBD-07-002</t>
-  </si>
-  <si>
-    <t>LIBD-07-003</t>
-  </si>
-  <si>
-    <t>E16°54'36.07"</t>
-  </si>
-  <si>
     <t>3 Nm from previous fix</t>
   </si>
   <si>
@@ -113,9 +98,6 @@
     <t>E16°57'00.89"</t>
   </si>
   <si>
-    <t>LIBD-07-004</t>
-  </si>
-  <si>
     <t>N41°04'48.12"</t>
   </si>
   <si>
@@ -125,21 +107,9 @@
     <t>5,78 Nm from previous fix</t>
   </si>
   <si>
-    <t>LIBD-07-005</t>
-  </si>
-  <si>
     <t>N41°01'55.55"</t>
   </si>
   <si>
-    <t>E16°56'58.31"</t>
-  </si>
-  <si>
-    <t>E16°50'19.19"</t>
-  </si>
-  <si>
-    <t>LIBD-07-006</t>
-  </si>
-  <si>
     <t>13,80 Nm from previous fix</t>
   </si>
   <si>
@@ -149,10 +119,55 @@
     <t>first fix of the route</t>
   </si>
   <si>
-    <t>E16°32'57.70"</t>
-  </si>
-  <si>
     <t>N41°06'2.27"</t>
+  </si>
+  <si>
+    <t>N41°31'48.99"</t>
+  </si>
+  <si>
+    <t>E016°38'10.99"</t>
+  </si>
+  <si>
+    <t>E016°51'11.30''</t>
+  </si>
+  <si>
+    <t>E016°54'36.07"</t>
+  </si>
+  <si>
+    <t>E016°56'58.31"</t>
+  </si>
+  <si>
+    <t>E016°50'19.19"</t>
+  </si>
+  <si>
+    <t>E016°32'57.70"</t>
+  </si>
+  <si>
+    <t>RWY-07-001</t>
+  </si>
+  <si>
+    <t>RWY-07-002</t>
+  </si>
+  <si>
+    <t>RWY-07-003</t>
+  </si>
+  <si>
+    <t>RWY-07-004</t>
+  </si>
+  <si>
+    <t>RWY-07-005</t>
+  </si>
+  <si>
+    <t>RWY-07-006</t>
+  </si>
+  <si>
+    <t>RWY-07-007</t>
+  </si>
+  <si>
+    <t>N41°01'33.00"</t>
+  </si>
+  <si>
+    <t>E016°40'07.00"</t>
   </si>
 </sst>
 </file>
@@ -530,12 +545,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4250DF5B-50B6-4ED2-A2AE-C2F89150E5A0}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.7265625" customWidth="1"/>
     <col min="3" max="3" width="26.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" customWidth="1"/>
+    <col min="4" max="4" width="25.453125" customWidth="1"/>
     <col min="5" max="5" width="13.26953125" customWidth="1"/>
     <col min="6" max="7" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
@@ -571,19 +586,19 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -591,22 +606,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
         <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -614,22 +629,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -637,22 +652,22 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -660,22 +675,22 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -683,22 +698,22 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -706,22 +721,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -729,13 +744,45 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
       </c>
       <c r="E9" t="s">
         <v>1</v>
       </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
       <c r="G9" t="s">
-        <v>35</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>